<commit_message>
feat: actualizar nómina y sincronizar presupuestos a requerimientos fase 1
</commit_message>
<xml_diff>
--- a/Estudios/Presupuestos/presupuesto_clinica_mejorado_13.xlsx
+++ b/Estudios/Presupuestos/presupuesto_clinica_mejorado_13.xlsx
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3374733.451</v>
+        <v>5041405.646000001</v>
       </c>
     </row>
     <row r="4">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5534733.451</v>
+        <v>7201405.646000001</v>
       </c>
     </row>
     <row r="5">
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3284733.451</v>
+        <v>4951405.646000001</v>
       </c>
     </row>
     <row r="7">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>21346794.451</v>
+        <v>23013466.646</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>33208400.706</v>
+        <v>43208433.876</v>
       </c>
     </row>
     <row r="9">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>54555195.157</v>
+        <v>66221900.522</v>
       </c>
     </row>
   </sheetData>
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1281,13 +1281,13 @@
         <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>910710.6</v>
+        <v>984649.4650000001</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>910710.6</v>
+        <v>984649.4650000001</v>
       </c>
     </row>
     <row r="32">
@@ -1305,13 +1305,13 @@
         <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>1310710.6</v>
+        <v>1884649.465</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>1310710.6</v>
+        <v>1884649.465</v>
       </c>
     </row>
     <row r="33">
@@ -1322,20 +1322,20 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Sueldo Técnico Fijo (Mes 1 Sincronizado)</t>
+          <t>Sueldo Médico 2 (Mes 1 Sincronizado)</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>812062.2509999999</v>
+        <v>880044.4650000001</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>812062.2509999999</v>
+        <v>880044.4650000001</v>
       </c>
     </row>
     <row r="34">
@@ -1346,20 +1346,20 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Sueldo Técnico Boleta (Mes 1 Sincronizado)</t>
+          <t>Sueldo Médico 3 (Mes 1 Sincronizado)</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>341250</v>
+        <v>300000</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>341250</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="35">
@@ -1370,20 +1370,20 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Internet</t>
+          <t>Sueldo Técnicos (Mes 1 Sincronizado)</t>
         </is>
       </c>
       <c r="C35" t="n">
         <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>27000</v>
+        <v>180000</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>27000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="36">
@@ -1394,20 +1394,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Insumos Hospital y Consulta</t>
+          <t>Sueldo Recepcionista 2 (Mes 1 Sincronizado)</t>
         </is>
       </c>
       <c r="C36" t="n">
         <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>1200000</v>
+        <v>812062.2509999999</v>
       </c>
       <c r="E36" t="n">
-        <v>228000</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>1428000</v>
+        <v>812062.2509999999</v>
       </c>
     </row>
     <row r="37">
@@ -1418,20 +1418,20 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Camara de seguridad x4</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="C37" t="n">
         <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>200000</v>
+        <v>27000</v>
       </c>
       <c r="E37" t="n">
-        <v>38000</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>238000</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="38">
@@ -1442,20 +1442,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Software + stack</t>
+          <t>Insumos Hospital y Consulta</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>300000</v>
+        <v>1200000</v>
       </c>
       <c r="E38" t="n">
-        <v>57000</v>
+        <v>228000</v>
       </c>
       <c r="F38" t="n">
-        <v>357000</v>
+        <v>1428000</v>
       </c>
     </row>
     <row r="39">
@@ -1466,44 +1466,92 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SEO Inicial</t>
+          <t>Camara de seguridad x4</t>
         </is>
       </c>
       <c r="C39" t="n">
         <v>1</v>
       </c>
       <c r="D39" t="n">
-        <v>1000000</v>
+        <v>200000</v>
       </c>
       <c r="E39" t="n">
-        <v>0</v>
+        <v>38000</v>
       </c>
       <c r="F39" t="n">
-        <v>1000000</v>
+        <v>238000</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>Costos Iniciales</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Software + stack</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E40" t="n">
+        <v>57000</v>
+      </c>
+      <c r="F40" t="n">
+        <v>357000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Costos Iniciales</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>SEO Inicial</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>Caja Seguridad</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>FONDO DE EMERGENCIA (6 Meses Costos Fijos)</t>
         </is>
       </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
-        <v>33208400.706</v>
-      </c>
-      <c r="E40" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" t="n">
-        <v>33208400.706</v>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>43208433.876</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>43208433.876</v>
       </c>
     </row>
   </sheetData>
@@ -1653,7 +1701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1674,12 +1722,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Retiro Mensual (Libre Imp.)</t>
+          <t>Retiro de Socia (Libre Imp.)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Ingreso Líquido Aprox (Bolsillo)</t>
+          <t>Ingreso Líquido (Bolsillo)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -1691,84 +1739,84 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sasha (Socia Administradora)</t>
+          <t>Daniela (Socia Directora Médica)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sueldo Patronal + Retiro</t>
+          <t>Contrato Trabajo + Retiro</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>553553</v>
+        <v>395395</v>
       </c>
       <c r="D2" t="n">
-        <v>246447</v>
+        <v>1304605</v>
       </c>
       <c r="E2" t="n">
-        <v>800000</v>
+        <v>1700000</v>
       </c>
       <c r="F2" t="n">
-        <v>910710.6</v>
+        <v>1884649.465</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Daniela (Socia Jefe Médico)</t>
+          <t>Sasha (Socia Recepción)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sueldo Patronal + Retiro</t>
+          <t>Contrato Trabajo + Retiro</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>553553</v>
+        <v>395395</v>
       </c>
       <c r="D3" t="n">
-        <v>646447</v>
+        <v>404605</v>
       </c>
       <c r="E3" t="n">
-        <v>1200000</v>
+        <v>800000</v>
       </c>
       <c r="F3" t="n">
-        <v>1310710.6</v>
+        <v>984649.4650000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Técnico Veterinario (Fijo)</t>
+          <t>Médico 2 (Tarde/Sábado)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Contrato Fijo (Con Aportes + Provisiones Ahorro)</t>
+          <t>Contrato Trabajo (Part-Time)</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>553553</v>
+        <v>395395</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>553553</v>
+        <v>695395</v>
       </c>
       <c r="F4" t="n">
-        <v>812062.2509999999</v>
+        <v>880044.4650000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Técnico (Boleta/Part-Time)</t>
+          <t>Médico 3 (Fines de semana)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Prestación de Servicios</t>
+          <t>Boleta Honorarios</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1778,10 +1826,58 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
+        <v>258750</v>
+      </c>
+      <c r="F5" t="n">
         <v>300000</v>
       </c>
-      <c r="F5" t="n">
-        <v>341250</v>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Técnicos (Diurno/Nocturno)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Boleta Honorarios</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>155250</v>
+      </c>
+      <c r="F6" t="n">
+        <v>180000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Recepcionista 2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Contrato Trabajo (Full-Time)</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>553553</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>553553</v>
+      </c>
+      <c r="F7" t="n">
+        <v>812062.2509999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(presupuesto): ajustar horas de medico 3 y tecnicos a 0 por ser 100% variables
</commit_message>
<xml_diff>
--- a/Estudios/Presupuestos/presupuesto_clinica_mejorado_13.xlsx
+++ b/Estudios/Presupuestos/presupuesto_clinica_mejorado_13.xlsx
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5041405.646000001</v>
+        <v>4561405.646000001</v>
       </c>
     </row>
     <row r="4">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7201405.646000001</v>
+        <v>6721405.646000001</v>
       </c>
     </row>
     <row r="5">
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4951405.646000001</v>
+        <v>4471405.646000001</v>
       </c>
     </row>
     <row r="7">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>23013466.646</v>
+        <v>22533466.646</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>43208433.876</v>
+        <v>40328433.876</v>
       </c>
     </row>
     <row r="9">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>66221900.522</v>
+        <v>62861900.522</v>
       </c>
     </row>
   </sheetData>
@@ -1353,13 +1353,13 @@
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>300000</v>
+        <v>0</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>300000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -1377,13 +1377,13 @@
         <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>180000</v>
+        <v>0</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>180000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -1545,13 +1545,13 @@
         <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>43208433.876</v>
+        <v>40328433.876</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>43208433.876</v>
+        <v>40328433.876</v>
       </c>
     </row>
   </sheetData>
@@ -1826,10 +1826,10 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>258750</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>300000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1850,10 +1850,10 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>155250</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>180000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
feat(docs,presupuesto): actualizar Estudio Máster a V13 e Inversión Total .2M
</commit_message>
<xml_diff>
--- a/Estudios/Presupuestos/presupuesto_clinica_mejorado_13.xlsx
+++ b/Estudios/Presupuestos/presupuesto_clinica_mejorado_13.xlsx
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4561405.646000001</v>
+        <v>5041405.646000001</v>
       </c>
     </row>
     <row r="4">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6721405.646000001</v>
+        <v>7201405.646000001</v>
       </c>
     </row>
     <row r="5">
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4471405.646000001</v>
+        <v>4951405.646000001</v>
       </c>
     </row>
     <row r="7">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>22533466.646</v>
+        <v>23013466.646</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>40328433.876</v>
+        <v>43208433.876</v>
       </c>
     </row>
     <row r="9">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>62861900.522</v>
+        <v>66221900.522</v>
       </c>
     </row>
   </sheetData>
@@ -1353,13 +1353,13 @@
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>300000</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="35">
@@ -1377,13 +1377,13 @@
         <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>180000</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="36">
@@ -1545,13 +1545,13 @@
         <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>40328433.876</v>
+        <v>43208433.876</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>40328433.876</v>
+        <v>43208433.876</v>
       </c>
     </row>
   </sheetData>
@@ -1826,10 +1826,10 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>258750</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="6">
@@ -1850,10 +1850,10 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>155250</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="7">

</xml_diff>